<commit_message>
Simplify station-first workflow and laptop layouts
</commit_message>
<xml_diff>
--- a/templates/站位表导入模板.xlsx
+++ b/templates/站位表导入模板.xlsx
@@ -11,7 +11,7 @@
     <sheet name="填写说明" sheetId="2" state="visible" r:id="rId2"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Worksheet'!$A$1:$C$2</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Worksheet'!$A$1:$B$2</definedName>
     <definedName name="_xlnm.Print_Titles" localSheetId="0">'Worksheet'!$1:$1</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -208,11 +208,6 @@
         <t>Example value - replace or delete this row before import.</t>
       </text>
     </comment>
-    <comment ref="C2" authorId="0" shapeId="0">
-      <text>
-        <t>Example value - replace or delete this row before import.</t>
-      </text>
-    </comment>
   </commentList>
 </comments>
 </file>
@@ -507,26 +502,20 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:C2"/>
+  <dimension ref="A1:B2"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
-    <col width="18" customWidth="1" min="1" max="1"/>
-    <col width="18" customWidth="1" min="2" max="2"/>
-    <col width="22" customWidth="1" min="3" max="3"/>
+    <col width="20" customWidth="1" min="1" max="1"/>
+    <col width="24" customWidth="1" min="2" max="2"/>
   </cols>
   <sheetData>
     <row r="1" ht="28" customHeight="1">
       <c r="A1" s="1" t="inlineStr">
         <is>
-          <t>设备编码</t>
+          <t>站位编码</t>
         </is>
       </c>
       <c r="B1" s="1" t="inlineStr">
-        <is>
-          <t>站位编码</t>
-        </is>
-      </c>
-      <c r="C1" s="1" t="inlineStr">
         <is>
           <t>物料编码</t>
         </is>
@@ -535,22 +524,17 @@
     <row r="2" ht="24" customHeight="1">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>SMT-01</t>
+          <t>F-01</t>
         </is>
       </c>
       <c r="B2" s="2" t="inlineStr">
-        <is>
-          <t>F-01</t>
-        </is>
-      </c>
-      <c r="C2" s="2" t="inlineStr">
         <is>
           <t>013000081</t>
         </is>
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A1:C2"/>
+  <autoFilter ref="A1:B2"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
   <pageSetup orientation="landscape" fitToHeight="0" fitToWidth="1"/>
   <legacyDrawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="anysvml"/>
@@ -605,7 +589,7 @@
     <row r="3">
       <c r="A3" s="5" t="inlineStr">
         <is>
-          <t>设备编码</t>
+          <t>站位编码</t>
         </is>
       </c>
       <c r="B3" s="5" t="inlineStr">
@@ -615,19 +599,19 @@
       </c>
       <c r="C3" s="5" t="inlineStr">
         <is>
-          <t>SMT-01</t>
+          <t>F-01</t>
         </is>
       </c>
       <c r="D3" s="5" t="inlineStr">
         <is>
-          <t>必须先在软件的“设备与站位”页面创建并启用</t>
+          <t>必须全局唯一，并已在“设备与站位”页面创建和启用</t>
         </is>
       </c>
     </row>
     <row r="4">
       <c r="A4" s="5" t="inlineStr">
         <is>
-          <t>站位编码</t>
+          <t>物料编码</t>
         </is>
       </c>
       <c r="B4" s="5" t="inlineStr">
@@ -637,34 +621,34 @@
       </c>
       <c r="C4" s="5" t="inlineStr">
         <is>
-          <t>F-01</t>
+          <t>013000081</t>
         </is>
       </c>
       <c r="D4" s="5" t="inlineStr">
         <is>
-          <t>必须属于对应设备并处于启用状态</t>
+          <t>按文本填写并保留前导零；不要求预先导入 BOM</t>
         </is>
       </c>
     </row>
     <row r="5">
       <c r="A5" s="5" t="inlineStr">
         <is>
-          <t>物料编码</t>
+          <t>设备编码</t>
         </is>
       </c>
       <c r="B5" s="5" t="inlineStr">
         <is>
-          <t>是</t>
+          <t>否</t>
         </is>
       </c>
       <c r="C5" s="5" t="inlineStr">
         <is>
-          <t>013000081</t>
+          <t>SMT-01</t>
         </is>
       </c>
       <c r="D5" s="5" t="inlineStr">
         <is>
-          <t>按文本填写，必须保留前导零并存在于已导入 BOM</t>
+          <t>仅兼容旧表；如填写，必须与该站位的所属设备一致</t>
         </is>
       </c>
     </row>

</xml_diff>